<commit_message>
Registra roles, hora de descarga y reemplazos de la calibración (E1 y E2)
- Registro de búsqueda: hora de descarga 21:54 (8 oct 2026) y responsable (MSC).
- Bitácora de decisiones: sección E con roles del equipo (MSC coordinador de datos) y sección D con los reemplazos de la selección de calibración.
- Checklist E1 y bitácora de etapas actualizados.
- Planillas y selección de calibración regeneradas con los 4 reemplazos.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X4evu4SUuSdB43CdCRdWEX
</commit_message>
<xml_diff>
--- a/data/calibracion/plantilla_codificacion_calibracion_EDU_JPM.xlsx
+++ b/data/calibracion/plantilla_codificacion_calibracion_EDU_JPM.xlsx
@@ -2435,22 +2435,22 @@
       </c>
       <c r="B8" s="27" t="inlineStr">
         <is>
-          <t>10.1080/14767724.2026.2673130</t>
+          <t>10.5209/rced.96906</t>
         </is>
       </c>
       <c r="C8" s="28" t="inlineStr">
         <is>
-          <t>Decolonial in theory, colonial in practice? Rethinking gatekeeping from within the Global South</t>
+          <t>Empowerment profiles in students with intellectual disabilities of the Todos Somos Campus University program</t>
         </is>
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>WOS:001765460900001</t>
+          <t>WOS:001589228100009</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
-          <t>GLOBALISATION SOCIETIES AND EDUCATION</t>
+          <t>REVISTA COMPLUTENSE DE EDUCACION</t>
         </is>
       </c>
       <c r="F8" s="29" t="n"/>
@@ -2635,22 +2635,22 @@
       </c>
       <c r="B10" s="27" t="inlineStr">
         <is>
-          <t>10.1108/JPCC-09-2024-0166</t>
+          <t>10.1007/s10639-024-13003-4</t>
         </is>
       </c>
       <c r="C10" s="28" t="inlineStr">
         <is>
-          <t>Understanding the role of structural capital as facilitator in professional learning networks and organizational learning of university</t>
+          <t>Efficient topic identification for urgent MOOC Forum posts using BERTopic and traditional topic modeling techniques</t>
         </is>
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>WOS:001572686000001</t>
+          <t>WOS:001314860800001</t>
         </is>
       </c>
       <c r="E10" s="27" t="inlineStr">
         <is>
-          <t>JOURNAL OF PROFESSIONAL CAPITAL AND COMMUNITY</t>
+          <t>EDUCATION AND INFORMATION TECHNOLOGIES</t>
         </is>
       </c>
       <c r="F10" s="29" t="n"/>
@@ -2835,22 +2835,22 @@
       </c>
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>10.1080/08841241.2022.2109093</t>
+          <t>10.1038/s41539-026-00405-x</t>
         </is>
       </c>
       <c r="C12" s="28" t="inlineStr">
         <is>
-          <t>Changing trends of rates of return: a study from the higher education market in China</t>
+          <t>A Bayesian perspective on observers' inference of group norms</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>WOS:000858989100001</t>
+          <t>WOS:001736040400001</t>
         </is>
       </c>
       <c r="E12" s="27" t="inlineStr">
         <is>
-          <t>JOURNAL OF MARKETING FOR HIGHER EDUCATION</t>
+          <t>NPJ SCIENCE OF LEARNING</t>
         </is>
       </c>
       <c r="F12" s="29" t="n"/>
@@ -3435,22 +3435,22 @@
       </c>
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>10.1080/00219266.2024.2420013</t>
+          <t>10.1186/s12909-025-07133-7</t>
         </is>
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>Development and validation of the Perspective Scale on the Origin of Life and Biodiversity (PSOLB)</t>
+          <t>Association of completing an intercalated year-long research degree with post-graduation academic success</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>WOS:001347489700001</t>
+          <t>WOS:001553695100004</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
         <is>
-          <t>JOURNAL OF BIOLOGICAL EDUCATION</t>
+          <t>BMC MEDICAL EDUCATION</t>
         </is>
       </c>
       <c r="F18" s="29" t="n"/>

</xml_diff>